<commit_message>
Rename the study to GLPX-1
</commit_message>
<xml_diff>
--- a/data/spec/SDTM_METADATA.xlsx
+++ b/data/spec/SDTM_METADATA.xlsx
@@ -49,13 +49,13 @@
     <t xml:space="preserve">STYLESHEET</t>
   </si>
   <si>
-    <t xml:space="preserve">GLPX001.define.sdtm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GLPX001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GLPX-001</t>
+    <t xml:space="preserve">GLPX1.define.sdtm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GLPX1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GLPX-1</t>
   </si>
   <si>
     <t xml:space="preserve">A simulated Phase III trial of GLPX 10 mg in type 2 diabetes</t>
@@ -1314,7 +1314,7 @@
         <v>55</v>
       </c>
       <c r="E2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F2" t="s">
         <v>56</v>
@@ -1388,7 +1388,7 @@
         <v>55</v>
       </c>
       <c r="E4" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F4" t="s">
         <v>60</v>
@@ -2264,7 +2264,7 @@
         <v>55</v>
       </c>
       <c r="E28" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F28" t="s">
         <v>56</v>
@@ -2338,7 +2338,7 @@
         <v>55</v>
       </c>
       <c r="E30" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F30" t="s">
         <v>60</v>

</xml_diff>